<commit_message>
analyzed IDX11 and IDX30. also fixed minor bugs to code
</commit_message>
<xml_diff>
--- a/NURBS IDX11 PYTHON ANALYSIS/8_4_2026_Redo_front/15gps/1mps_15gps_analysis.xlsx
+++ b/NURBS IDX11 PYTHON ANALYSIS/8_4_2026_Redo_front/15gps/1mps_15gps_analysis.xlsx
@@ -691,7 +691,7 @@
         <v>0</v>
       </c>
       <c r="W3">
-        <v>247.9420662470201</v>
+        <v>248.2541260715633</v>
       </c>
       <c r="X3">
         <v>0.253114294</v>
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="W5">
-        <v>23.5612009976136</v>
+        <v>23.56858304551885</v>
       </c>
       <c r="X5">
         <v>0.253077418</v>
@@ -1729,7 +1729,7 @@
         <v>246.2591981035281</v>
       </c>
       <c r="V15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X15">
         <v>0.252966154</v>
@@ -1815,7 +1815,7 @@
         <v>244.9913844121824</v>
       </c>
       <c r="V16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X16">
         <v>0.252976962</v>
@@ -1901,7 +1901,7 @@
         <v>244.755962480199</v>
       </c>
       <c r="V17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X17">
         <v>0.252964246</v>
@@ -1987,7 +1987,7 @@
         <v>244.2155064840763</v>
       </c>
       <c r="V18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X18">
         <v>0.252953756</v>

</xml_diff>